<commit_message>
Add SOH report for 2026-10-06
</commit_message>
<xml_diff>
--- a/reports/SOH_05_10_2026.xlsx
+++ b/reports/SOH_05_10_2026.xlsx
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>2</v>
+        <v>-4</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>8000</v>
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>21000</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>2</v>
+        <v>-16</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>8000</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1121</v>
+        <v>1112</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>40000</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>490</v>
+        <v>480</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>10500</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>653</v>
+        <v>647</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>589</v>
+        <v>580</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1356</v>
+        <v>1340</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>869</v>
+        <v>852</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>983</v>
+        <v>977</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>3000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -3009,7 +3009,7 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="E92" s="3" t="n">
         <v>8000</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>975</v>
+        <v>909</v>
       </c>
       <c r="E93" s="3" t="n">
         <v>8000</v>
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="E95" s="3" t="n">
         <v>7612</v>
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="E98" s="3" t="n">
         <v>8597</v>
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="E99" s="3" t="n">
         <v>8597</v>
@@ -3233,7 +3233,7 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E100" s="3" t="n">
         <v>8597</v>
@@ -3261,7 +3261,7 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E101" s="3" t="n">
         <v>8597</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>4708</v>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E104" s="3" t="n">
         <v>4708</v>
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E119" s="3" t="n">
         <v>5000</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2421</v>
+        <v>2331</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>4950</v>
+        <v>4926</v>
       </c>
       <c r="E126" s="3" t="n">
         <v>2500</v>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>886</v>
+        <v>838</v>
       </c>
       <c r="E128" s="3" t="n">
         <v>3500</v>
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="E129" s="3" t="n">
         <v>2500</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>1661</v>
+        <v>1655</v>
       </c>
       <c r="E140" s="3" t="n">
         <v>7845</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>505</v>
+        <v>493</v>
       </c>
       <c r="E174" s="3" t="n">
         <v>13500</v>
@@ -5445,7 +5445,7 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>1811</v>
+        <v>811</v>
       </c>
       <c r="E180" s="3" t="n">
         <v>0</v>
@@ -7945,7 +7945,7 @@
         </is>
       </c>
       <c r="D272" s="2" t="n">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="E272" s="3" t="n">
         <v>5648</v>
@@ -7973,7 +7973,7 @@
         </is>
       </c>
       <c r="D273" s="2" t="n">
-        <v>478</v>
+        <v>430</v>
       </c>
       <c r="E273" s="3" t="n">
         <v>5308</v>
@@ -8001,7 +8001,7 @@
         </is>
       </c>
       <c r="D274" s="2" t="n">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="E274" s="3" t="n">
         <v>3954</v>
@@ -8057,7 +8057,7 @@
         </is>
       </c>
       <c r="D276" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E276" s="3" t="n">
         <v>3614</v>
@@ -8505,7 +8505,7 @@
         </is>
       </c>
       <c r="D292" s="2" t="n">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E292" s="3" t="n">
         <v>80577</v>
@@ -8617,7 +8617,7 @@
         </is>
       </c>
       <c r="D296" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E296" s="3" t="n">
         <v>12281</v>
@@ -9177,7 +9177,7 @@
         </is>
       </c>
       <c r="D316" s="2" t="n">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="E316" s="3" t="n">
         <v>39894</v>
@@ -9373,7 +9373,7 @@
         </is>
       </c>
       <c r="D323" s="2" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E323" s="3" t="n">
         <v>10962</v>
@@ -9906,7 +9906,7 @@
         </is>
       </c>
       <c r="D342" s="2" t="n">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="E342" s="3" t="n">
         <v>6251</v>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="D346" s="2" t="n">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E346" s="3" t="n">
         <v>10439</v>
@@ -10382,7 +10382,7 @@
         </is>
       </c>
       <c r="D359" s="2" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E359" s="3" t="n">
         <v>16261</v>
@@ -12650,7 +12650,7 @@
         </is>
       </c>
       <c r="D440" s="2" t="n">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E440" s="3" t="n">
         <v>9967</v>
@@ -13098,7 +13098,7 @@
         </is>
       </c>
       <c r="D456" s="2" t="n">
-        <v>866</v>
+        <v>818</v>
       </c>
       <c r="E456" s="3" t="n">
         <v>9621</v>
@@ -13126,7 +13126,7 @@
         </is>
       </c>
       <c r="D457" s="2" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E457" s="3" t="n">
         <v>7235</v>
@@ -13378,7 +13378,7 @@
         </is>
       </c>
       <c r="D466" s="2" t="n">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="E466" s="3" t="n">
         <v>13959</v>
@@ -14414,7 +14414,7 @@
         </is>
       </c>
       <c r="D503" s="2" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E503" s="3" t="n">
         <v>3672</v>
@@ -14498,7 +14498,7 @@
         </is>
       </c>
       <c r="D506" s="2" t="n">
-        <v>1281</v>
+        <v>1257</v>
       </c>
       <c r="E506" s="3" t="n">
         <v>8446</v>
@@ -14666,7 +14666,7 @@
         </is>
       </c>
       <c r="D512" s="2" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E512" s="3" t="n">
         <v>68040</v>
@@ -14862,7 +14862,7 @@
         </is>
       </c>
       <c r="D519" s="2" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E519" s="3" t="n">
         <v>12900</v>
@@ -14946,7 +14946,7 @@
         </is>
       </c>
       <c r="D522" s="2" t="n">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="E522" s="3" t="n">
         <v>13237</v>
@@ -15114,7 +15114,7 @@
         </is>
       </c>
       <c r="D528" s="2" t="n">
-        <v>463</v>
+        <v>445</v>
       </c>
       <c r="E528" s="3" t="n">
         <v>22302</v>
@@ -15170,7 +15170,7 @@
         </is>
       </c>
       <c r="D530" s="2" t="n">
-        <v>394</v>
+        <v>370</v>
       </c>
       <c r="E530" s="3" t="n">
         <v>12816</v>
@@ -15338,7 +15338,7 @@
         </is>
       </c>
       <c r="D536" s="2" t="n">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="E536" s="3" t="n">
         <v>30244</v>
@@ -15534,7 +15534,7 @@
         </is>
       </c>
       <c r="D543" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E543" s="3" t="n">
         <v>11000</v>
@@ -15926,7 +15926,7 @@
         </is>
       </c>
       <c r="D557" s="2" t="n">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E557" s="3" t="n">
         <v>10491</v>
@@ -16094,7 +16094,7 @@
         </is>
       </c>
       <c r="D563" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E563" s="3" t="n">
         <v>10840</v>
@@ -16150,7 +16150,7 @@
         </is>
       </c>
       <c r="D565" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E565" s="3" t="n">
         <v>8752</v>
@@ -16570,7 +16570,7 @@
         </is>
       </c>
       <c r="D580" s="2" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E580" s="3" t="n">
         <v>18839</v>
@@ -16598,7 +16598,7 @@
         </is>
       </c>
       <c r="D581" s="2" t="n">
-        <v>1181</v>
+        <v>1175</v>
       </c>
       <c r="E581" s="3" t="n">
         <v>19364</v>
@@ -17242,7 +17242,7 @@
         </is>
       </c>
       <c r="D604" s="2" t="n">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="E604" s="3" t="n">
         <v>8331</v>
@@ -17327,7 +17327,7 @@
         </is>
       </c>
       <c r="D607" s="2" t="n">
-        <v>491</v>
+        <v>467</v>
       </c>
       <c r="E607" s="3" t="n">
         <v>7801</v>
@@ -17551,7 +17551,7 @@
         </is>
       </c>
       <c r="D615" s="2" t="n">
-        <v>4403</v>
+        <v>4379</v>
       </c>
       <c r="E615" s="3" t="n">
         <v>10251</v>
@@ -17579,7 +17579,7 @@
         </is>
       </c>
       <c r="D616" s="2" t="n">
-        <v>488</v>
+        <v>464</v>
       </c>
       <c r="E616" s="3" t="n">
         <v>12094</v>
@@ -17775,7 +17775,7 @@
         </is>
       </c>
       <c r="D623" s="2" t="n">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E623" s="3" t="n">
         <v>12330</v>
@@ -17803,7 +17803,7 @@
         </is>
       </c>
       <c r="D624" s="2" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E624" s="3" t="n">
         <v>10030</v>
@@ -17887,7 +17887,7 @@
         </is>
       </c>
       <c r="D627" s="2" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E627" s="3" t="n">
         <v>21996</v>
@@ -18559,7 +18559,7 @@
         </is>
       </c>
       <c r="D651" s="2" t="n">
-        <v>886</v>
+        <v>862</v>
       </c>
       <c r="E651" s="3" t="n">
         <v>6417</v>
@@ -18615,7 +18615,7 @@
         </is>
       </c>
       <c r="D653" s="2" t="n">
-        <v>1177</v>
+        <v>1153</v>
       </c>
       <c r="E653" s="3" t="n">
         <v>11078</v>
@@ -18895,7 +18895,7 @@
         </is>
       </c>
       <c r="D663" s="2" t="n">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E663" s="3" t="n">
         <v>3987</v>
@@ -19343,7 +19343,7 @@
         </is>
       </c>
       <c r="D679" s="2" t="n">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="E679" s="3" t="n">
         <v>2338</v>
@@ -19987,7 +19987,7 @@
         </is>
       </c>
       <c r="D702" s="2" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E702" s="3" t="n">
         <v>4213</v>
@@ -20211,7 +20211,7 @@
         </is>
       </c>
       <c r="D710" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E710" s="3" t="n">
         <v>9818</v>
@@ -20379,7 +20379,7 @@
         </is>
       </c>
       <c r="D716" s="2" t="n">
-        <v>475</v>
+        <v>463</v>
       </c>
       <c r="E716" s="3" t="n">
         <v>5340</v>
@@ -21191,7 +21191,7 @@
         </is>
       </c>
       <c r="D745" s="2" t="n">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E745" s="3" t="n">
         <v>9853</v>
@@ -21219,7 +21219,7 @@
         </is>
       </c>
       <c r="D746" s="2" t="n">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="E746" s="3" t="n">
         <v>5157</v>
@@ -21415,7 +21415,7 @@
         </is>
       </c>
       <c r="D753" s="2" t="n">
-        <v>209</v>
+        <v>185</v>
       </c>
       <c r="E753" s="3" t="n">
         <v>6440</v>
@@ -21751,7 +21751,7 @@
         </is>
       </c>
       <c r="D765" s="2" t="n">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="E765" s="3" t="n">
         <v>6934</v>
@@ -21779,7 +21779,7 @@
         </is>
       </c>
       <c r="D766" s="2" t="n">
-        <v>731</v>
+        <v>695</v>
       </c>
       <c r="E766" s="3" t="n">
         <v>7465</v>
@@ -21919,7 +21919,7 @@
         </is>
       </c>
       <c r="D771" s="2" t="n">
-        <v>856</v>
+        <v>844</v>
       </c>
       <c r="E771" s="3" t="n">
         <v>3731</v>
@@ -22031,7 +22031,7 @@
         </is>
       </c>
       <c r="D775" s="2" t="n">
-        <v>628</v>
+        <v>616</v>
       </c>
       <c r="E775" s="3" t="n">
         <v>15899</v>
@@ -22199,7 +22199,7 @@
         </is>
       </c>
       <c r="D781" s="2" t="n">
-        <v>422</v>
+        <v>386</v>
       </c>
       <c r="E781" s="3" t="n">
         <v>7016</v>
@@ -23207,7 +23207,7 @@
         </is>
       </c>
       <c r="D817" s="2" t="n">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="E817" s="3" t="n">
         <v>16983</v>
@@ -23880,7 +23880,7 @@
         </is>
       </c>
       <c r="D841" s="2" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E841" s="3" t="n">
         <v>13122</v>
@@ -23908,7 +23908,7 @@
         </is>
       </c>
       <c r="D842" s="2" t="n">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E842" s="3" t="n">
         <v>34247</v>
@@ -24637,7 +24637,7 @@
         </is>
       </c>
       <c r="D868" s="2" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E868" s="3" t="n">
         <v>9047</v>
@@ -24721,7 +24721,7 @@
         </is>
       </c>
       <c r="D871" s="2" t="n">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="E871" s="3" t="n">
         <v>14083</v>
@@ -26096,7 +26096,7 @@
         </is>
       </c>
       <c r="D920" s="2" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E920" s="3" t="n">
         <v>8700</v>
@@ -28168,7 +28168,7 @@
         </is>
       </c>
       <c r="D994" s="2" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E994" s="3" t="n">
         <v>23590</v>
@@ -28560,7 +28560,7 @@
         </is>
       </c>
       <c r="D1008" s="2" t="n">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="E1008" s="3" t="n">
         <v>9408</v>
@@ -28868,7 +28868,7 @@
         </is>
       </c>
       <c r="D1019" s="2" t="n">
-        <v>234</v>
+        <v>210</v>
       </c>
       <c r="E1019" s="3" t="n">
         <v>8060</v>
@@ -29316,7 +29316,7 @@
         </is>
       </c>
       <c r="D1035" s="2" t="n">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="E1035" s="3" t="n">
         <v>10809</v>
@@ -29485,7 +29485,7 @@
         </is>
       </c>
       <c r="D1041" s="2" t="n">
-        <v>388</v>
+        <v>352</v>
       </c>
       <c r="E1041" s="3" t="n">
         <v>9527</v>
@@ -29849,7 +29849,7 @@
         </is>
       </c>
       <c r="D1054" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E1054" s="3" t="n">
         <v>32068</v>
@@ -30129,7 +30129,7 @@
         </is>
       </c>
       <c r="D1064" s="2" t="n">
-        <v>581</v>
+        <v>569</v>
       </c>
       <c r="E1064" s="3" t="n">
         <v>3247</v>
@@ -30437,7 +30437,7 @@
         </is>
       </c>
       <c r="D1075" s="2" t="n">
-        <v>550</v>
+        <v>538</v>
       </c>
       <c r="E1075" s="3" t="n">
         <v>9226</v>
@@ -30773,7 +30773,7 @@
         </is>
       </c>
       <c r="D1087" s="2" t="n">
-        <v>1185</v>
+        <v>1161</v>
       </c>
       <c r="E1087" s="3" t="n">
         <v>5086</v>
@@ -31305,7 +31305,7 @@
         </is>
       </c>
       <c r="D1106" s="2" t="n">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="E1106" s="3" t="n">
         <v>11372</v>
@@ -32201,7 +32201,7 @@
         </is>
       </c>
       <c r="D1138" s="2" t="n">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="E1138" s="3" t="n">
         <v>4651</v>
@@ -32397,7 +32397,7 @@
         </is>
       </c>
       <c r="D1145" s="2" t="n">
-        <v>193</v>
+        <v>169</v>
       </c>
       <c r="E1145" s="3" t="n">
         <v>14752</v>
@@ -32425,7 +32425,7 @@
         </is>
       </c>
       <c r="D1146" s="2" t="n">
-        <v>776</v>
+        <v>770</v>
       </c>
       <c r="E1146" s="3" t="n">
         <v>6111</v>
@@ -32761,7 +32761,7 @@
         </is>
       </c>
       <c r="D1158" s="2" t="n">
-        <v>345</v>
+        <v>321</v>
       </c>
       <c r="E1158" s="3" t="n">
         <v>9174</v>
@@ -33013,7 +33013,7 @@
         </is>
       </c>
       <c r="D1167" s="2" t="n">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="E1167" s="3" t="n">
         <v>13001</v>
@@ -33041,7 +33041,7 @@
         </is>
       </c>
       <c r="D1168" s="2" t="n">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="E1168" s="3" t="n">
         <v>11269</v>
@@ -33321,7 +33321,7 @@
         </is>
       </c>
       <c r="D1178" s="2" t="n">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="E1178" s="3" t="n">
         <v>14554</v>
@@ -33769,7 +33769,7 @@
         </is>
       </c>
       <c r="D1194" s="2" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E1194" s="3" t="n">
         <v>12500</v>
@@ -33965,7 +33965,7 @@
         </is>
       </c>
       <c r="D1201" s="2" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E1201" s="3" t="n">
         <v>5601</v>
@@ -34133,7 +34133,7 @@
         </is>
       </c>
       <c r="D1207" s="2" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E1207" s="3" t="n">
         <v>6594</v>
@@ -34665,7 +34665,7 @@
         </is>
       </c>
       <c r="D1226" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E1226" s="3" t="n">
         <v>89163</v>
@@ -35533,7 +35533,7 @@
         </is>
       </c>
       <c r="D1257" s="2" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E1257" s="3" t="n">
         <v>36976</v>
@@ -35701,7 +35701,7 @@
         </is>
       </c>
       <c r="D1263" s="2" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E1263" s="3" t="n">
         <v>13998</v>
@@ -36317,7 +36317,7 @@
         </is>
       </c>
       <c r="D1285" s="2" t="n">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="E1285" s="3" t="n">
         <v>24210</v>
@@ -37045,7 +37045,7 @@
         </is>
       </c>
       <c r="D1311" s="2" t="n">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E1311" s="3" t="n">
         <v>8781</v>
@@ -37381,7 +37381,7 @@
         </is>
       </c>
       <c r="D1323" s="2" t="n">
-        <v>733</v>
+        <v>709</v>
       </c>
       <c r="E1323" s="3" t="n">
         <v>10365</v>
@@ -37437,7 +37437,7 @@
         </is>
       </c>
       <c r="D1325" s="2" t="n">
-        <v>1516</v>
+        <v>1492</v>
       </c>
       <c r="E1325" s="3" t="n">
         <v>10295</v>
@@ -37605,7 +37605,7 @@
         </is>
       </c>
       <c r="D1331" s="2" t="n">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="E1331" s="3" t="n">
         <v>13995</v>
@@ -37913,7 +37913,7 @@
         </is>
       </c>
       <c r="D1342" s="2" t="n">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="E1342" s="3" t="n">
         <v>3137</v>
@@ -38137,7 +38137,7 @@
         </is>
       </c>
       <c r="D1350" s="2" t="n">
-        <v>1370</v>
+        <v>1358</v>
       </c>
       <c r="E1350" s="3" t="n">
         <v>14093</v>
@@ -38725,7 +38725,7 @@
         </is>
       </c>
       <c r="D1371" s="2" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E1371" s="3" t="n">
         <v>30208</v>
@@ -39593,7 +39593,7 @@
         </is>
       </c>
       <c r="D1402" s="2" t="n">
-        <v>240</v>
+        <v>192</v>
       </c>
       <c r="E1402" s="3" t="n">
         <v>5837</v>
@@ -39677,7 +39677,7 @@
         </is>
       </c>
       <c r="D1405" s="2" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="E1405" s="3" t="n">
         <v>9007</v>
@@ -40209,7 +40209,7 @@
         </is>
       </c>
       <c r="D1424" s="2" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E1424" s="3" t="n">
         <v>16220</v>
@@ -40349,7 +40349,7 @@
         </is>
       </c>
       <c r="D1429" s="2" t="n">
-        <v>778</v>
+        <v>766</v>
       </c>
       <c r="E1429" s="3" t="n">
         <v>3140</v>
@@ -40657,7 +40657,7 @@
         </is>
       </c>
       <c r="D1440" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E1440" s="3" t="n">
         <v>10733</v>
@@ -40741,7 +40741,7 @@
         </is>
       </c>
       <c r="D1443" s="2" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="E1443" s="3" t="n">
         <v>5153</v>
@@ -41217,7 +41217,7 @@
         </is>
       </c>
       <c r="D1460" s="2" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E1460" s="3" t="n">
         <v>9428</v>
@@ -41245,7 +41245,7 @@
         </is>
       </c>
       <c r="D1461" s="2" t="n">
-        <v>383</v>
+        <v>359</v>
       </c>
       <c r="E1461" s="3" t="n">
         <v>11283</v>
@@ -41553,7 +41553,7 @@
         </is>
       </c>
       <c r="D1472" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="E1472" s="3" t="n">
         <v>4836</v>
@@ -41581,7 +41581,7 @@
         </is>
       </c>
       <c r="D1473" s="2" t="n">
-        <v>2650</v>
+        <v>2626</v>
       </c>
       <c r="E1473" s="3" t="n">
         <v>7312</v>
@@ -41749,7 +41749,7 @@
         </is>
       </c>
       <c r="D1479" s="2" t="n">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E1479" s="3" t="n">
         <v>7390</v>
@@ -41833,7 +41833,7 @@
         </is>
       </c>
       <c r="D1482" s="2" t="n">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="E1482" s="3" t="n">
         <v>11171</v>
@@ -42337,7 +42337,7 @@
         </is>
       </c>
       <c r="D1500" s="2" t="n">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E1500" s="3" t="n">
         <v>19321</v>
@@ -42421,7 +42421,7 @@
         </is>
       </c>
       <c r="D1503" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E1503" s="3" t="n">
         <v>12491</v>
@@ -43066,7 +43066,7 @@
         </is>
       </c>
       <c r="D1526" s="2" t="n">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E1526" s="3" t="n">
         <v>6639</v>
@@ -43430,7 +43430,7 @@
         </is>
       </c>
       <c r="D1539" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E1539" s="3" t="n">
         <v>10405</v>
@@ -43907,7 +43907,7 @@
         </is>
       </c>
       <c r="D1556" s="2" t="n">
-        <v>541</v>
+        <v>517</v>
       </c>
       <c r="E1556" s="3" t="n">
         <v>4577</v>
@@ -44047,7 +44047,7 @@
         </is>
       </c>
       <c r="D1561" s="2" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E1561" s="3" t="n">
         <v>23136</v>

</xml_diff>